<commit_message>
Add cDNA as suspension entity type
Closes #149
</commit_message>
<xml_diff>
--- a/sample-suspension/latest/sample-suspension.xlsx
+++ b/sample-suspension/latest/sample-suspension.xlsx
@@ -178,7 +178,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="226" uniqueCount="174">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="230" uniqueCount="176">
   <si>
     <t>source_id</t>
   </si>
@@ -498,6 +498,12 @@
     <t>http://ncicb.nci.nih.gov/xml/owl/EVS/Thesaurus.owl#C185338</t>
   </si>
   <si>
+    <t>Incubated at 37 degrees celsius</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000148</t>
+  </si>
+  <si>
     <t>Frozen at -20 degrees celsius</t>
   </si>
   <si>
@@ -618,12 +624,6 @@
     <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000387</t>
   </si>
   <si>
-    <t>Incubated at 37 degrees celsius</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000148</t>
-  </si>
-  <si>
     <t>Frozen at -80 degrees celsius</t>
   </si>
   <si>
@@ -648,6 +648,12 @@
     <t>http://ncicb.nci.nih.gov/xml/owl/EVS/Thesaurus.owl#C13197</t>
   </si>
   <si>
+    <t>cDNA</t>
+  </si>
+  <si>
+    <t>http://ncicb.nci.nih.gov/xml/owl/EVS/Thesaurus.owl#C324</t>
+  </si>
+  <si>
     <t>Cell</t>
   </si>
   <si>
@@ -693,7 +699,7 @@
     <t>pav:createdOn</t>
   </si>
   <si>
-    <t>2026-02-24T15:31:04-08:00</t>
+    <t>2026-03-06T11:08:03-08:00</t>
   </si>
   <si>
     <t>pav:derivedFrom</t>
@@ -846,16 +852,16 @@
         <v>97</v>
       </c>
       <c r="K1" t="s" s="1">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="L1" t="s" s="1">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="M1" t="s" s="1">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="N1" t="s" s="1">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="O1" t="s" s="1">
         <v>150</v>
@@ -864,24 +870,24 @@
         <v>151</v>
       </c>
       <c r="Q1" t="s" s="1">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="R1" t="s" s="1">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="S1" t="s" s="1">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="T1" t="s" s="1">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="U1" t="s" s="1">
-        <v>164</v>
+        <v>166</v>
       </c>
     </row>
     <row r="2">
       <c r="U2" t="s" s="22">
-        <v>165</v>
+        <v>167</v>
       </c>
     </row>
   </sheetData>
@@ -904,7 +910,7 @@
       <formula1>'preparation_medium'!$A$1:$A$35</formula1>
     </dataValidation>
     <dataValidation type="list" sqref="J2:J1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="" showErrorMessage="true">
-      <formula1>'preparation_condition'!$A$1:$A$9</formula1>
+      <formula1>'preparation_condition'!$A$1:$A$10</formula1>
     </dataValidation>
     <dataValidation type="decimal" operator="greaterThanOrEqual" sqref="K2:K1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="Value should be greater than 0" showErrorMessage="true">
       <formula1>0</formula1>
@@ -920,7 +926,7 @@
       <formula1>'storage_method'!$A$1:$A$12</formula1>
     </dataValidation>
     <dataValidation type="list" sqref="P2:P1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="" showErrorMessage="true">
-      <formula1>'suspension_entity_type'!$A$1:$A$3</formula1>
+      <formula1>'suspension_entity_type'!$A$1:$A$4</formula1>
     </dataValidation>
     <dataValidation type="whole" operator="greaterThanOrEqual" sqref="Q2:Q1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="Value should be greater than 0" showErrorMessage="true">
       <formula1>0</formula1>
@@ -943,12 +949,12 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="0">
-        <v>160</v>
+        <v>162</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s" s="0">
-        <v>161</v>
+        <v>163</v>
       </c>
     </row>
   </sheetData>
@@ -969,30 +975,30 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="0">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B1" t="s" s="0">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="C1" t="s" s="0">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="D1" t="s" s="0">
-        <v>172</v>
+        <v>174</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s" s="0">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="C2" t="s" s="0">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="D2" t="s" s="0">
-        <v>173</v>
+        <v>175</v>
       </c>
     </row>
   </sheetData>
@@ -1384,7 +1390,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -1457,6 +1463,14 @@
       </c>
       <c r="B9" t="s" s="0">
         <v>113</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s" s="0">
+        <v>114</v>
+      </c>
+      <c r="B10" t="s" s="0">
+        <v>115</v>
       </c>
     </row>
   </sheetData>
@@ -1505,18 +1519,18 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="0">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="B1" t="s" s="0">
-        <v>118</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s" s="0">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>120</v>
+        <v>122</v>
       </c>
     </row>
     <row r="3">
@@ -1537,10 +1551,10 @@
     </row>
     <row r="5">
       <c r="A5" t="s" s="0">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="B5" t="s" s="0">
-        <v>122</v>
+        <v>124</v>
       </c>
     </row>
     <row r="6">
@@ -1561,34 +1575,34 @@
     </row>
     <row r="8">
       <c r="A8" t="s" s="0">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="B8" t="s" s="0">
-        <v>124</v>
+        <v>126</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s" s="0">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="B9" t="s" s="0">
-        <v>126</v>
+        <v>128</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s" s="0">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B10" t="s" s="0">
-        <v>128</v>
+        <v>130</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s" s="0">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="B11" t="s" s="0">
-        <v>130</v>
+        <v>132</v>
       </c>
     </row>
     <row r="12">
@@ -1625,10 +1639,10 @@
     </row>
     <row r="16">
       <c r="A16" t="s" s="0">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B16" t="s" s="0">
-        <v>132</v>
+        <v>134</v>
       </c>
     </row>
     <row r="17">
@@ -1641,10 +1655,10 @@
     </row>
     <row r="18">
       <c r="A18" t="s" s="0">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="B18" t="s" s="0">
-        <v>134</v>
+        <v>136</v>
       </c>
     </row>
     <row r="19">
@@ -1665,26 +1679,26 @@
     </row>
     <row r="21">
       <c r="A21" t="s" s="0">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="B21" t="s" s="0">
-        <v>136</v>
+        <v>138</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s" s="0">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="B22" t="s" s="0">
-        <v>138</v>
+        <v>140</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s" s="0">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B23" t="s" s="0">
-        <v>140</v>
+        <v>142</v>
       </c>
     </row>
     <row r="24">
@@ -1697,10 +1711,10 @@
     </row>
     <row r="25">
       <c r="A25" t="s" s="0">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="B25" t="s" s="0">
-        <v>142</v>
+        <v>144</v>
       </c>
     </row>
     <row r="26">
@@ -1763,18 +1777,18 @@
     </row>
     <row r="6">
       <c r="A6" t="s" s="0">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="B6" t="s" s="0">
-        <v>145</v>
+        <v>147</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s" s="0">
-        <v>146</v>
+        <v>106</v>
       </c>
       <c r="B7" t="s" s="0">
-        <v>147</v>
+        <v>107</v>
       </c>
     </row>
     <row r="8">
@@ -1787,26 +1801,26 @@
     </row>
     <row r="9">
       <c r="A9" t="s" s="0">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="B9" t="s" s="0">
-        <v>107</v>
+        <v>109</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s" s="0">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B10" t="s" s="0">
-        <v>109</v>
+        <v>111</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s" s="0">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="B11" t="s" s="0">
-        <v>111</v>
+        <v>113</v>
       </c>
     </row>
     <row r="12">
@@ -1824,7 +1838,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:B4"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -1851,6 +1865,14 @@
         <v>157</v>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="s" s="0">
+        <v>158</v>
+      </c>
+      <c r="B4" t="s" s="0">
+        <v>159</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>